<commit_message>
fix: Robust signer name replacement in all templates
</commit_message>
<xml_diff>
--- a/data sample/DATA SAMPLE THANG/9.HIỆN TRẠNG THIẾT BỊ_TÂM.xlsx
+++ b/data sample/DATA SAMPLE THANG/9.HIỆN TRẠNG THIẾT BỊ_TÂM.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\quyng\Documents\TOOL TỔNG HỢP BÁO CÁO\VNPT REPORT\data sample\DATA SAMPLE THANG\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56092C64-DE2B-45D7-BA79-6B7567816BB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8BE4C2F-313C-4BEC-A8B5-12F9E05377F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-24" yWindow="12852" windowWidth="23256" windowHeight="12456" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="01_MANE_CSG" sheetId="1" r:id="rId1"/>
@@ -227,25 +227,25 @@
     <t>Vĩnh Hưng</t>
   </si>
   <si>
-    <t>B1</t>
-  </si>
-  <si>
-    <t>B2</t>
-  </si>
-  <si>
-    <t>B3</t>
-  </si>
-  <si>
-    <t>B4</t>
-  </si>
-  <si>
-    <t>B5</t>
-  </si>
-  <si>
-    <t>B6</t>
-  </si>
-  <si>
-    <t>B7</t>
+    <t>B1_TAM</t>
+  </si>
+  <si>
+    <t>B2_TAM</t>
+  </si>
+  <si>
+    <t>B3_TAM</t>
+  </si>
+  <si>
+    <t>B4_TAM</t>
+  </si>
+  <si>
+    <t>B5_TAM</t>
+  </si>
+  <si>
+    <t>B6_TAM</t>
+  </si>
+  <si>
+    <t>B7_TAM</t>
   </si>
 </sst>
 </file>
@@ -638,7 +638,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:J11"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
@@ -646,7 +646,7 @@
     <col min="7" max="9" width="15" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="18.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" ht="18" x14ac:dyDescent="0.3">
       <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
@@ -662,7 +662,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
@@ -691,7 +691,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>10</v>
       </c>
@@ -707,7 +707,9 @@
       <c r="E4" s="2">
         <v>47</v>
       </c>
-      <c r="F4" s="2"/>
+      <c r="F4" s="2">
+        <v>47</v>
+      </c>
       <c r="G4" s="2">
         <v>48</v>
       </c>
@@ -718,7 +720,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A5" s="2">
         <v>1</v>
       </c>
@@ -734,7 +736,9 @@
       <c r="E5" s="2">
         <v>10</v>
       </c>
-      <c r="F5" s="2"/>
+      <c r="F5" s="2">
+        <v>10</v>
+      </c>
       <c r="G5" s="2">
         <v>7</v>
       </c>
@@ -745,7 +749,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A6" s="2">
         <v>2</v>
       </c>
@@ -761,7 +765,9 @@
       <c r="E6" s="2">
         <v>8</v>
       </c>
-      <c r="F6" s="2"/>
+      <c r="F6" s="2">
+        <v>8</v>
+      </c>
       <c r="G6" s="2">
         <v>7</v>
       </c>
@@ -772,7 +778,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A7" s="2">
         <v>3</v>
       </c>
@@ -788,7 +794,9 @@
       <c r="E7" s="2">
         <v>5</v>
       </c>
-      <c r="F7" s="2"/>
+      <c r="F7" s="2">
+        <v>5</v>
+      </c>
       <c r="G7" s="2">
         <v>8</v>
       </c>
@@ -799,7 +807,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A8" s="2">
         <v>4</v>
       </c>
@@ -815,7 +823,9 @@
       <c r="E8" s="2">
         <v>2</v>
       </c>
-      <c r="F8" s="2"/>
+      <c r="F8" s="2">
+        <v>2</v>
+      </c>
       <c r="G8" s="2">
         <v>5</v>
       </c>
@@ -826,7 +836,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A9" s="2">
         <v>5</v>
       </c>
@@ -842,7 +852,9 @@
       <c r="E9" s="2">
         <v>13</v>
       </c>
-      <c r="F9" s="2"/>
+      <c r="F9" s="2">
+        <v>13</v>
+      </c>
       <c r="G9" s="2">
         <v>6</v>
       </c>
@@ -853,7 +865,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A10" s="2">
         <v>6</v>
       </c>
@@ -869,7 +881,9 @@
       <c r="E10" s="2">
         <v>4</v>
       </c>
-      <c r="F10" s="2"/>
+      <c r="F10" s="2">
+        <v>4</v>
+      </c>
       <c r="G10" s="2">
         <v>9</v>
       </c>
@@ -880,7 +894,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A11" s="2">
         <v>7</v>
       </c>
@@ -896,7 +910,9 @@
       <c r="E11" s="2">
         <v>5</v>
       </c>
-      <c r="F11" s="2"/>
+      <c r="F11" s="2">
+        <v>5</v>
+      </c>
       <c r="G11" s="2">
         <v>6</v>
       </c>
@@ -920,7 +936,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:H11"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
@@ -928,7 +944,7 @@
     <col min="4" max="7" width="13" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="18.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" ht="18" x14ac:dyDescent="0.3">
       <c r="A1" s="6" t="s">
         <v>19</v>
       </c>
@@ -942,7 +958,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
@@ -965,7 +981,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>10</v>
       </c>
@@ -986,7 +1002,7 @@
       </c>
       <c r="G4" s="2"/>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" s="2">
         <v>1</v>
       </c>
@@ -1007,7 +1023,7 @@
       </c>
       <c r="G5" s="2"/>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" s="2">
         <v>2</v>
       </c>
@@ -1028,7 +1044,7 @@
       </c>
       <c r="G6" s="2"/>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A7" s="2">
         <v>3</v>
       </c>
@@ -1049,7 +1065,7 @@
       </c>
       <c r="G7" s="2"/>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8" s="2">
         <v>4</v>
       </c>
@@ -1070,7 +1086,7 @@
       </c>
       <c r="G8" s="2"/>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A9" s="2">
         <v>5</v>
       </c>
@@ -1091,7 +1107,7 @@
       </c>
       <c r="G9" s="2"/>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A10" s="2">
         <v>6</v>
       </c>
@@ -1112,7 +1128,7 @@
       </c>
       <c r="G10" s="2"/>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A11" s="2">
         <v>7</v>
       </c>
@@ -1146,7 +1162,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:G11"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
@@ -1154,7 +1170,7 @@
     <col min="4" max="6" width="13" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="18.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" ht="18" x14ac:dyDescent="0.3">
       <c r="A1" s="6" t="s">
         <v>26</v>
       </c>
@@ -1167,7 +1183,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
@@ -1187,7 +1203,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>10</v>
       </c>
@@ -1207,7 +1223,7 @@
         <v>838</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" s="2">
         <v>1</v>
       </c>
@@ -1227,7 +1243,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" s="2">
         <v>2</v>
       </c>
@@ -1247,7 +1263,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" s="2">
         <v>3</v>
       </c>
@@ -1267,7 +1283,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" s="2">
         <v>4</v>
       </c>
@@ -1287,7 +1303,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" s="2">
         <v>5</v>
       </c>
@@ -1307,7 +1323,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" s="2">
         <v>6</v>
       </c>
@@ -1327,7 +1343,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" s="2">
         <v>7</v>
       </c>
@@ -1360,18 +1376,18 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:B6"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
     <col min="2" max="2" width="100" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" ht="18" x14ac:dyDescent="0.35">
       <c r="A1" s="4" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" s="5" t="s">
         <v>29</v>
       </c>
@@ -1379,7 +1395,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" s="5" t="s">
         <v>31</v>
       </c>
@@ -1387,7 +1403,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" s="5" t="s">
         <v>33</v>
       </c>
@@ -1395,7 +1411,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" s="5" t="s">
         <v>35</v>
       </c>
@@ -1412,7 +1428,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:G11"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
@@ -1420,7 +1436,7 @@
     <col min="4" max="6" width="13" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="18.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" ht="18" x14ac:dyDescent="0.3">
       <c r="A1" s="6" t="s">
         <v>37</v>
       </c>
@@ -1433,7 +1449,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
@@ -1453,7 +1469,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>10</v>
       </c>
@@ -1473,7 +1489,7 @@
         <v>1638</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" s="2">
         <v>1</v>
       </c>
@@ -1493,7 +1509,7 @@
         <v>240</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" s="2">
         <v>2</v>
       </c>
@@ -1513,7 +1529,7 @@
         <v>276</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" s="2">
         <v>3</v>
       </c>
@@ -1533,7 +1549,7 @@
         <v>223</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" s="2">
         <v>4</v>
       </c>
@@ -1553,7 +1569,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" s="2">
         <v>5</v>
       </c>
@@ -1573,7 +1589,7 @@
         <v>224</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" s="2">
         <v>6</v>
       </c>
@@ -1593,7 +1609,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" s="2">
         <v>7</v>
       </c>
@@ -1626,7 +1642,7 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:G11"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
@@ -1634,7 +1650,7 @@
     <col min="4" max="6" width="13" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="18.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" ht="18" x14ac:dyDescent="0.3">
       <c r="A1" s="6" t="s">
         <v>39</v>
       </c>
@@ -1647,7 +1663,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
@@ -1667,7 +1683,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>10</v>
       </c>
@@ -1687,7 +1703,7 @@
         <v>1901</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" s="2">
         <v>1</v>
       </c>
@@ -1707,7 +1723,7 @@
         <v>256</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" s="2">
         <v>2</v>
       </c>
@@ -1727,7 +1743,7 @@
         <v>403</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" s="2">
         <v>3</v>
       </c>
@@ -1747,7 +1763,7 @@
         <v>251</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" s="2">
         <v>4</v>
       </c>
@@ -1767,7 +1783,7 @@
         <v>241</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" s="2">
         <v>5</v>
       </c>
@@ -1787,7 +1803,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" s="2">
         <v>6</v>
       </c>
@@ -1807,7 +1823,7 @@
         <v>265</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" s="2">
         <v>7</v>
       </c>
@@ -1840,7 +1856,7 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:G11"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
@@ -1848,7 +1864,7 @@
     <col min="4" max="6" width="13" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="18.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" ht="18" x14ac:dyDescent="0.3">
       <c r="A1" s="6" t="s">
         <v>41</v>
       </c>
@@ -1861,7 +1877,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
@@ -1881,7 +1897,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>10</v>
       </c>
@@ -1901,7 +1917,7 @@
         <v>215</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" s="2">
         <v>1</v>
       </c>
@@ -1921,7 +1937,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" s="2">
         <v>2</v>
       </c>
@@ -1941,7 +1957,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" s="2">
         <v>3</v>
       </c>
@@ -1961,7 +1977,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" s="2">
         <v>4</v>
       </c>
@@ -1981,7 +1997,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" s="2">
         <v>5</v>
       </c>
@@ -2001,7 +2017,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" s="2">
         <v>6</v>
       </c>
@@ -2021,7 +2037,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" s="2">
         <v>7</v>
       </c>
@@ -2054,7 +2070,7 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1:G26"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
     <col min="2" max="2" width="20" customWidth="1"/>
@@ -2062,7 +2078,7 @@
     <col min="4" max="6" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="18.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" ht="18" x14ac:dyDescent="0.3">
       <c r="A1" s="6" t="s">
         <v>43</v>
       </c>
@@ -2075,7 +2091,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
@@ -2095,7 +2111,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>10</v>
       </c>
@@ -2115,7 +2131,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" s="2">
         <v>1</v>
       </c>
@@ -2135,7 +2151,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" s="2">
         <v>2</v>
       </c>
@@ -2155,7 +2171,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" s="2">
         <v>3</v>
       </c>
@@ -2175,7 +2191,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" s="2">
         <v>4</v>
       </c>
@@ -2195,7 +2211,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" s="2">
         <v>5</v>
       </c>
@@ -2215,7 +2231,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" s="2">
         <v>6</v>
       </c>
@@ -2235,7 +2251,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" s="2">
         <v>7</v>
       </c>
@@ -2255,7 +2271,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A12" s="2">
         <v>8</v>
       </c>
@@ -2275,7 +2291,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13" s="2">
         <v>9</v>
       </c>
@@ -2295,7 +2311,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A14" s="2">
         <v>10</v>
       </c>
@@ -2315,7 +2331,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A15" s="2">
         <v>11</v>
       </c>
@@ -2335,7 +2351,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A16" s="2">
         <v>12</v>
       </c>
@@ -2355,7 +2371,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A17" s="2">
         <v>13</v>
       </c>
@@ -2375,7 +2391,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A18" s="2">
         <v>14</v>
       </c>
@@ -2395,7 +2411,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A19" s="2">
         <v>15</v>
       </c>
@@ -2415,7 +2431,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A20" s="2">
         <v>16</v>
       </c>
@@ -2435,7 +2451,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A21" s="2">
         <v>17</v>
       </c>
@@ -2455,7 +2471,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A22" s="2">
         <v>18</v>
       </c>
@@ -2475,7 +2491,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A23" s="2">
         <v>19</v>
       </c>
@@ -2495,7 +2511,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A24" s="2">
         <v>20</v>
       </c>
@@ -2515,7 +2531,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A25" s="2">
         <v>21</v>
       </c>
@@ -2535,7 +2551,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A26" s="2">
         <v>22</v>
       </c>

</xml_diff>